<commit_message>
ajuste na meta novembro
</commit_message>
<xml_diff>
--- a/data/meta_marcas_televendas.xlsx
+++ b/data/meta_marcas_televendas.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\convenção\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9E18AC8-6E62-4399-8706-A059625F08F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153EB97A-1B1A-4F81-AA16-43F2FC9D9A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="2850" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MARCA E." sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MARCA E.'!$B$1:$D$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MARCA E.'!$A$1:$E$154</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="9">
   <si>
     <t>DATA</t>
   </si>
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -172,6 +172,24 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -478,11 +496,11 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E204"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="5"/>
-    <col min="2" max="2" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" style="7" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36" style="8" bestFit="1" customWidth="1"/>
@@ -1378,15 +1396,15 @@
         <v>1</v>
       </c>
       <c r="B53" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C53" s="6">
-        <v>27</v>
+        <v>1139</v>
       </c>
       <c r="D53" s="3">
-        <v>15000</v>
-      </c>
-      <c r="E53" s="5" t="s">
+        <v>30000</v>
+      </c>
+      <c r="E53" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1395,15 +1413,15 @@
         <v>1</v>
       </c>
       <c r="B54" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C54" s="6">
-        <v>1139</v>
+        <v>675</v>
       </c>
       <c r="D54" s="3">
-        <v>30000</v>
-      </c>
-      <c r="E54" s="5" t="s">
+        <v>7000</v>
+      </c>
+      <c r="E54" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1412,15 +1430,15 @@
         <v>1</v>
       </c>
       <c r="B55" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C55" s="6">
-        <v>675</v>
+        <v>58</v>
       </c>
       <c r="D55" s="3">
         <v>7000</v>
       </c>
-      <c r="E55" s="5" t="s">
+      <c r="E55" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1429,15 +1447,15 @@
         <v>1</v>
       </c>
       <c r="B56" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C56" s="6">
-        <v>58</v>
+        <v>841</v>
       </c>
       <c r="D56" s="3">
         <v>7000</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="E56" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1446,15 +1464,15 @@
         <v>1</v>
       </c>
       <c r="B57" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C57" s="6">
-        <v>841</v>
+        <v>13148</v>
       </c>
       <c r="D57" s="3">
         <v>7000</v>
       </c>
-      <c r="E57" s="5" t="s">
+      <c r="E57" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1463,15 +1481,15 @@
         <v>1</v>
       </c>
       <c r="B58" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C58" s="6">
-        <v>13148</v>
+        <v>805</v>
       </c>
       <c r="D58" s="3">
-        <v>7000</v>
-      </c>
-      <c r="E58" s="5" t="s">
+        <v>17000</v>
+      </c>
+      <c r="E58" s="8" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1480,33 +1498,33 @@
         <v>1</v>
       </c>
       <c r="B59" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C59" s="6">
-        <v>805</v>
+        <v>3403</v>
       </c>
       <c r="D59" s="3">
-        <v>21000</v>
-      </c>
-      <c r="E59" s="5" t="s">
+        <v>10000</v>
+      </c>
+      <c r="E59" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B60" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C60" s="6">
-        <v>3403</v>
+        <v>1898</v>
       </c>
       <c r="D60" s="3">
-        <v>13000</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>2</v>
+        <v>16000</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1514,15 +1532,15 @@
         <v>2</v>
       </c>
       <c r="B61" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C61" s="6">
-        <v>1898</v>
+        <v>546</v>
       </c>
       <c r="D61" s="3">
-        <v>37500</v>
-      </c>
-      <c r="E61" s="5" t="s">
+        <v>20000</v>
+      </c>
+      <c r="E61" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1531,15 +1549,15 @@
         <v>2</v>
       </c>
       <c r="B62" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C62" s="6">
-        <v>546</v>
+        <v>422</v>
       </c>
       <c r="D62" s="3">
-        <v>20500</v>
-      </c>
-      <c r="E62" s="5" t="s">
+        <v>20000</v>
+      </c>
+      <c r="E62" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1548,15 +1566,15 @@
         <v>2</v>
       </c>
       <c r="B63" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C63" s="6">
-        <v>422</v>
+        <v>1281</v>
       </c>
       <c r="D63" s="3">
-        <v>39000</v>
-      </c>
-      <c r="E63" s="5" t="s">
+        <v>20000</v>
+      </c>
+      <c r="E63" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1565,15 +1583,15 @@
         <v>2</v>
       </c>
       <c r="B64" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C64" s="6">
-        <v>1281</v>
+        <v>2220</v>
       </c>
       <c r="D64" s="3">
-        <v>39000</v>
-      </c>
-      <c r="E64" s="5" t="s">
+        <v>14000</v>
+      </c>
+      <c r="E64" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1582,13 +1600,13 @@
         <v>2</v>
       </c>
       <c r="B65" s="1">
-        <v>46235</v>
+        <v>46204</v>
       </c>
       <c r="C65" s="6">
-        <v>2220</v>
+        <v>2571</v>
       </c>
       <c r="D65" s="3">
-        <v>34000</v>
+        <v>18000</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>1</v>
@@ -1596,33 +1614,33 @@
     </row>
     <row r="66" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5">
-        <v>2</v>
-      </c>
-      <c r="B66" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C66" s="6">
-        <v>2571</v>
-      </c>
-      <c r="D66" s="3">
-        <v>34000</v>
+        <v>3</v>
+      </c>
+      <c r="B66" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C66" s="16">
+        <v>2845</v>
+      </c>
+      <c r="D66" s="18">
+        <v>7000</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5">
         <v>3</v>
       </c>
-      <c r="B67" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C67" s="6">
-        <v>2845</v>
-      </c>
-      <c r="D67" s="3">
-        <v>10000</v>
+      <c r="B67" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C67" s="16">
+        <v>691</v>
+      </c>
+      <c r="D67" s="18">
+        <v>20000</v>
       </c>
       <c r="E67" s="8" t="s">
         <v>2</v>
@@ -1632,14 +1650,14 @@
       <c r="A68" s="5">
         <v>3</v>
       </c>
-      <c r="B68" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C68" s="6">
-        <v>691</v>
-      </c>
-      <c r="D68" s="3">
-        <v>21000</v>
+      <c r="B68" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C68" s="16">
+        <v>1533</v>
+      </c>
+      <c r="D68" s="18">
+        <v>22000</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>2</v>
@@ -1649,14 +1667,14 @@
       <c r="A69" s="5">
         <v>3</v>
       </c>
-      <c r="B69" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C69" s="6">
-        <v>1533</v>
-      </c>
-      <c r="D69" s="3">
-        <v>26000</v>
+      <c r="B69" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C69" s="16">
+        <v>738</v>
+      </c>
+      <c r="D69" s="18">
+        <v>20000</v>
       </c>
       <c r="E69" s="8" t="s">
         <v>2</v>
@@ -1666,14 +1684,14 @@
       <c r="A70" s="5">
         <v>3</v>
       </c>
-      <c r="B70" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C70" s="6">
-        <v>738</v>
-      </c>
-      <c r="D70" s="3">
-        <v>18000</v>
+      <c r="B70" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C70" s="16">
+        <v>213</v>
+      </c>
+      <c r="D70" s="18">
+        <v>13000</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>2</v>
@@ -1683,14 +1701,14 @@
       <c r="A71" s="5">
         <v>3</v>
       </c>
-      <c r="B71" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C71" s="6">
-        <v>213</v>
-      </c>
-      <c r="D71" s="3">
-        <v>60000</v>
+      <c r="B71" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C71" s="16">
+        <v>3009</v>
+      </c>
+      <c r="D71" s="18">
+        <v>18000</v>
       </c>
       <c r="E71" s="8" t="s">
         <v>2</v>
@@ -1698,33 +1716,33 @@
     </row>
     <row r="72" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5">
-        <v>3</v>
-      </c>
-      <c r="B72" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C72" s="6">
-        <v>3009</v>
-      </c>
-      <c r="D72" s="3">
-        <v>35000</v>
+        <v>4</v>
+      </c>
+      <c r="B72" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C72" s="16">
+        <v>3449</v>
+      </c>
+      <c r="D72" s="18">
+        <v>45000</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5">
         <v>4</v>
       </c>
-      <c r="B73" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C73" s="6">
-        <v>3449</v>
-      </c>
-      <c r="D73" s="3">
-        <v>52000</v>
+      <c r="B73" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C73" s="16">
+        <v>1953</v>
+      </c>
+      <c r="D73" s="18">
+        <v>45000</v>
       </c>
       <c r="E73" s="8" t="s">
         <v>1</v>
@@ -1734,14 +1752,14 @@
       <c r="A74" s="5">
         <v>4</v>
       </c>
-      <c r="B74" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C74" s="6">
-        <v>1953</v>
-      </c>
-      <c r="D74" s="3">
-        <v>42000</v>
+      <c r="B74" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C74" s="16">
+        <v>2853</v>
+      </c>
+      <c r="D74" s="18">
+        <v>40000</v>
       </c>
       <c r="E74" s="8" t="s">
         <v>1</v>
@@ -1749,16 +1767,16 @@
     </row>
     <row r="75" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5">
-        <v>4</v>
-      </c>
-      <c r="B75" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C75" s="6">
-        <v>2853</v>
-      </c>
-      <c r="D75" s="3">
-        <v>52000</v>
+        <v>5</v>
+      </c>
+      <c r="B75" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C75" s="16">
+        <v>977</v>
+      </c>
+      <c r="D75" s="18">
+        <v>18000</v>
       </c>
       <c r="E75" s="8" t="s">
         <v>1</v>
@@ -1768,14 +1786,14 @@
       <c r="A76" s="5">
         <v>5</v>
       </c>
-      <c r="B76" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C76" s="6">
-        <v>977</v>
-      </c>
-      <c r="D76" s="3">
-        <v>22500</v>
+      <c r="B76" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C76" s="16">
+        <v>423</v>
+      </c>
+      <c r="D76" s="18">
+        <v>16000</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>1</v>
@@ -1785,14 +1803,14 @@
       <c r="A77" s="5">
         <v>5</v>
       </c>
-      <c r="B77" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C77" s="6">
-        <v>423</v>
-      </c>
-      <c r="D77" s="3">
-        <v>20500</v>
+      <c r="B77" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C77" s="16">
+        <v>672</v>
+      </c>
+      <c r="D77" s="18">
+        <v>18000</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>1</v>
@@ -1802,14 +1820,14 @@
       <c r="A78" s="5">
         <v>5</v>
       </c>
-      <c r="B78" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C78" s="6">
-        <v>672</v>
-      </c>
-      <c r="D78" s="3">
-        <v>18000</v>
+      <c r="B78" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C78" s="16">
+        <v>1929</v>
+      </c>
+      <c r="D78" s="18">
+        <v>14000</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>1</v>
@@ -1819,14 +1837,14 @@
       <c r="A79" s="5">
         <v>5</v>
       </c>
-      <c r="B79" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C79" s="6">
-        <v>1929</v>
-      </c>
-      <c r="D79" s="3">
-        <v>17000</v>
+      <c r="B79" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C79" s="16">
+        <v>1087</v>
+      </c>
+      <c r="D79" s="18">
+        <v>16000</v>
       </c>
       <c r="E79" s="8" t="s">
         <v>1</v>
@@ -1836,14 +1854,14 @@
       <c r="A80" s="5">
         <v>5</v>
       </c>
-      <c r="B80" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C80" s="6">
-        <v>1087</v>
-      </c>
-      <c r="D80" s="3">
-        <v>20500</v>
+      <c r="B80" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C80" s="16">
+        <v>3179</v>
+      </c>
+      <c r="D80" s="18">
+        <v>14000</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>1</v>
@@ -1851,16 +1869,16 @@
     </row>
     <row r="81" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5">
-        <v>5</v>
-      </c>
-      <c r="B81" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C81" s="6">
-        <v>3179</v>
-      </c>
-      <c r="D81" s="3">
-        <v>16500</v>
+        <v>6</v>
+      </c>
+      <c r="B81" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C81" s="16">
+        <v>1954</v>
+      </c>
+      <c r="D81" s="18">
+        <v>35000</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>1</v>
@@ -1870,14 +1888,14 @@
       <c r="A82" s="5">
         <v>6</v>
       </c>
-      <c r="B82" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C82" s="6">
-        <v>1954</v>
-      </c>
-      <c r="D82" s="3">
-        <v>84000</v>
+      <c r="B82" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C82" s="16">
+        <v>1312</v>
+      </c>
+      <c r="D82" s="18">
+        <v>40000</v>
       </c>
       <c r="E82" s="8" t="s">
         <v>1</v>
@@ -1887,14 +1905,14 @@
       <c r="A83" s="5">
         <v>6</v>
       </c>
-      <c r="B83" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C83" s="6">
-        <v>1312</v>
-      </c>
-      <c r="D83" s="3">
-        <v>47000</v>
+      <c r="B83" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C83" s="16">
+        <v>874</v>
+      </c>
+      <c r="D83" s="18">
+        <v>40000</v>
       </c>
       <c r="E83" s="8" t="s">
         <v>1</v>
@@ -1902,33 +1920,33 @@
     </row>
     <row r="84" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5">
-        <v>6</v>
-      </c>
-      <c r="B84" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C84" s="6">
-        <v>874</v>
-      </c>
-      <c r="D84" s="3">
-        <v>94000</v>
+        <v>7</v>
+      </c>
+      <c r="B84" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C84" s="16">
+        <v>1899</v>
+      </c>
+      <c r="D84" s="18">
+        <v>15000</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="5">
         <v>7</v>
       </c>
-      <c r="B85" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C85" s="6">
-        <v>1899</v>
-      </c>
-      <c r="D85" s="3">
-        <v>15000</v>
+      <c r="B85" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C85" s="16">
+        <v>2985</v>
+      </c>
+      <c r="D85" s="18">
+        <v>10000</v>
       </c>
       <c r="E85" s="8" t="s">
         <v>3</v>
@@ -1938,14 +1956,14 @@
       <c r="A86" s="5">
         <v>7</v>
       </c>
-      <c r="B86" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C86" s="6">
-        <v>2985</v>
-      </c>
-      <c r="D86" s="3">
-        <v>10000</v>
+      <c r="B86" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C86" s="16">
+        <v>2184</v>
+      </c>
+      <c r="D86" s="18">
+        <v>15000</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>3</v>
@@ -1955,14 +1973,14 @@
       <c r="A87" s="5">
         <v>7</v>
       </c>
-      <c r="B87" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C87" s="6">
-        <v>2184</v>
-      </c>
-      <c r="D87" s="3">
-        <v>15000</v>
+      <c r="B87" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C87" s="16">
+        <v>519</v>
+      </c>
+      <c r="D87" s="18">
+        <v>20000</v>
       </c>
       <c r="E87" s="8" t="s">
         <v>3</v>
@@ -1972,14 +1990,14 @@
       <c r="A88" s="5">
         <v>7</v>
       </c>
-      <c r="B88" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C88" s="6">
-        <v>519</v>
-      </c>
-      <c r="D88" s="3">
-        <v>20000</v>
+      <c r="B88" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C88" s="16">
+        <v>2183</v>
+      </c>
+      <c r="D88" s="18">
+        <v>10000</v>
       </c>
       <c r="E88" s="8" t="s">
         <v>3</v>
@@ -1989,14 +2007,14 @@
       <c r="A89" s="5">
         <v>7</v>
       </c>
-      <c r="B89" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C89" s="6">
-        <v>2183</v>
-      </c>
-      <c r="D89" s="3">
-        <v>10000</v>
+      <c r="B89" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C89" s="16">
+        <v>1884</v>
+      </c>
+      <c r="D89" s="18">
+        <v>16000</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>3</v>
@@ -2006,14 +2024,14 @@
       <c r="A90" s="5">
         <v>7</v>
       </c>
-      <c r="B90" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C90" s="6">
-        <v>1884</v>
-      </c>
-      <c r="D90" s="3">
-        <v>16000</v>
+      <c r="B90" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C90" s="16">
+        <v>2185</v>
+      </c>
+      <c r="D90" s="18">
+        <v>10000</v>
       </c>
       <c r="E90" s="8" t="s">
         <v>3</v>
@@ -2023,14 +2041,14 @@
       <c r="A91" s="5">
         <v>7</v>
       </c>
-      <c r="B91" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C91" s="6">
-        <v>2185</v>
-      </c>
-      <c r="D91" s="3">
-        <v>10000</v>
+      <c r="B91" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C91" s="16">
+        <v>1885</v>
+      </c>
+      <c r="D91" s="18">
+        <v>13000</v>
       </c>
       <c r="E91" s="8" t="s">
         <v>3</v>
@@ -2040,14 +2058,14 @@
       <c r="A92" s="5">
         <v>7</v>
       </c>
-      <c r="B92" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C92" s="6">
-        <v>1885</v>
-      </c>
-      <c r="D92" s="3">
-        <v>13000</v>
+      <c r="B92" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C92" s="16">
+        <v>3389</v>
+      </c>
+      <c r="D92" s="18">
+        <v>8000</v>
       </c>
       <c r="E92" s="8" t="s">
         <v>3</v>
@@ -2057,14 +2075,14 @@
       <c r="A93" s="5">
         <v>7</v>
       </c>
-      <c r="B93" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C93" s="6">
-        <v>3389</v>
-      </c>
-      <c r="D93" s="3">
-        <v>8000</v>
+      <c r="B93" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C93" s="16">
+        <v>1883</v>
+      </c>
+      <c r="D93" s="18">
+        <v>12000</v>
       </c>
       <c r="E93" s="8" t="s">
         <v>3</v>
@@ -2072,33 +2090,33 @@
     </row>
     <row r="94" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5">
-        <v>7</v>
-      </c>
-      <c r="B94" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C94" s="6">
-        <v>1883</v>
-      </c>
-      <c r="D94" s="3">
-        <v>16000</v>
+        <v>9</v>
+      </c>
+      <c r="B94" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C94" s="16">
+        <v>2476</v>
+      </c>
+      <c r="D94" s="18">
+        <v>1490</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5">
         <v>9</v>
       </c>
-      <c r="B95" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C95" s="6">
-        <v>2476</v>
-      </c>
-      <c r="D95" s="3">
-        <v>1490</v>
+      <c r="B95" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C95" s="16">
+        <v>2494</v>
+      </c>
+      <c r="D95" s="18">
+        <v>1412</v>
       </c>
       <c r="E95" s="8" t="s">
         <v>4</v>
@@ -2108,14 +2126,14 @@
       <c r="A96" s="5">
         <v>9</v>
       </c>
-      <c r="B96" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C96" s="6">
-        <v>2494</v>
-      </c>
-      <c r="D96" s="3">
-        <v>1412</v>
+      <c r="B96" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C96" s="16">
+        <v>2661</v>
+      </c>
+      <c r="D96" s="18">
+        <v>1257</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>4</v>
@@ -2125,14 +2143,14 @@
       <c r="A97" s="5">
         <v>9</v>
       </c>
-      <c r="B97" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C97" s="6">
-        <v>2661</v>
-      </c>
-      <c r="D97" s="3">
-        <v>1257</v>
+      <c r="B97" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C97" s="16">
+        <v>3465</v>
+      </c>
+      <c r="D97" s="18">
+        <v>714</v>
       </c>
       <c r="E97" s="8" t="s">
         <v>4</v>
@@ -2142,13 +2160,13 @@
       <c r="A98" s="5">
         <v>9</v>
       </c>
-      <c r="B98" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C98" s="6">
-        <v>3465</v>
-      </c>
-      <c r="D98" s="3">
+      <c r="B98" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C98" s="16">
+        <v>1133</v>
+      </c>
+      <c r="D98" s="18">
         <v>714</v>
       </c>
       <c r="E98" s="8" t="s">
@@ -2159,13 +2177,13 @@
       <c r="A99" s="5">
         <v>9</v>
       </c>
-      <c r="B99" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C99" s="6">
-        <v>1133</v>
-      </c>
-      <c r="D99" s="3">
+      <c r="B99" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C99" s="16">
+        <v>3467</v>
+      </c>
+      <c r="D99" s="18">
         <v>714</v>
       </c>
       <c r="E99" s="8" t="s">
@@ -2174,16 +2192,16 @@
     </row>
     <row r="100" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5">
-        <v>9</v>
-      </c>
-      <c r="B100" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C100" s="6">
-        <v>3467</v>
-      </c>
-      <c r="D100" s="3">
-        <v>714</v>
+        <v>8</v>
+      </c>
+      <c r="B100" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C100" s="16">
+        <v>1762</v>
+      </c>
+      <c r="D100" s="18">
+        <v>42853</v>
       </c>
       <c r="E100" s="8" t="s">
         <v>4</v>
@@ -2193,14 +2211,14 @@
       <c r="A101" s="5">
         <v>8</v>
       </c>
-      <c r="B101" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C101" s="6">
-        <v>1762</v>
-      </c>
-      <c r="D101" s="3">
-        <v>42853</v>
+      <c r="B101" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C101" s="16">
+        <v>1778</v>
+      </c>
+      <c r="D101" s="18">
+        <v>40707</v>
       </c>
       <c r="E101" s="8" t="s">
         <v>4</v>
@@ -2210,14 +2228,14 @@
       <c r="A102" s="5">
         <v>8</v>
       </c>
-      <c r="B102" s="1">
-        <v>46235</v>
-      </c>
-      <c r="C102" s="6">
-        <v>1778</v>
-      </c>
-      <c r="D102" s="3">
-        <v>33671</v>
+      <c r="B102" s="14">
+        <v>46204</v>
+      </c>
+      <c r="C102" s="16">
+        <v>2727</v>
+      </c>
+      <c r="D102" s="18">
+        <v>39634</v>
       </c>
       <c r="E102" s="8" t="s">
         <v>4</v>
@@ -2225,19 +2243,19 @@
     </row>
     <row r="103" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B103" s="1">
         <v>46235</v>
       </c>
       <c r="C103" s="6">
-        <v>2727</v>
+        <v>27</v>
       </c>
       <c r="D103" s="3">
-        <v>29079</v>
-      </c>
-      <c r="E103" s="8" t="s">
-        <v>4</v>
+        <v>15000</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2245,15 +2263,15 @@
         <v>1</v>
       </c>
       <c r="B104" s="1">
-        <v>46266</v>
+        <v>46235</v>
       </c>
       <c r="C104" s="6">
-        <v>27</v>
+        <v>1139</v>
       </c>
       <c r="D104" s="3">
-        <v>15000</v>
-      </c>
-      <c r="E104" s="8" t="s">
+        <v>30000</v>
+      </c>
+      <c r="E104" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2262,15 +2280,15 @@
         <v>1</v>
       </c>
       <c r="B105" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C105" s="6">
-        <v>1139</v>
+        <v>675</v>
       </c>
       <c r="D105" s="3">
-        <v>30000</v>
-      </c>
-      <c r="E105" s="8" t="s">
+        <v>7000</v>
+      </c>
+      <c r="E105" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2279,15 +2297,15 @@
         <v>1</v>
       </c>
       <c r="B106" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C106" s="6">
-        <v>675</v>
+        <v>58</v>
       </c>
       <c r="D106" s="3">
         <v>7000</v>
       </c>
-      <c r="E106" s="8" t="s">
+      <c r="E106" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2296,15 +2314,15 @@
         <v>1</v>
       </c>
       <c r="B107" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C107" s="6">
-        <v>58</v>
+        <v>841</v>
       </c>
       <c r="D107" s="3">
         <v>7000</v>
       </c>
-      <c r="E107" s="8" t="s">
+      <c r="E107" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2313,15 +2331,15 @@
         <v>1</v>
       </c>
       <c r="B108" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C108" s="6">
-        <v>841</v>
+        <v>13148</v>
       </c>
       <c r="D108" s="3">
         <v>7000</v>
       </c>
-      <c r="E108" s="8" t="s">
+      <c r="E108" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2330,15 +2348,15 @@
         <v>1</v>
       </c>
       <c r="B109" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C109" s="6">
-        <v>13148</v>
+        <v>805</v>
       </c>
       <c r="D109" s="3">
-        <v>7000</v>
-      </c>
-      <c r="E109" s="8" t="s">
+        <v>21000</v>
+      </c>
+      <c r="E109" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -2347,33 +2365,33 @@
         <v>1</v>
       </c>
       <c r="B110" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C110" s="6">
-        <v>805</v>
+        <v>3403</v>
       </c>
       <c r="D110" s="3">
-        <v>17000</v>
-      </c>
-      <c r="E110" s="8" t="s">
+        <v>13000</v>
+      </c>
+      <c r="E110" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B111" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C111" s="6">
-        <v>3403</v>
+        <v>1898</v>
       </c>
       <c r="D111" s="3">
-        <v>10000</v>
-      </c>
-      <c r="E111" s="8" t="s">
-        <v>2</v>
+        <v>37500</v>
+      </c>
+      <c r="E111" s="5" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2381,15 +2399,15 @@
         <v>2</v>
       </c>
       <c r="B112" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C112" s="6">
-        <v>1898</v>
+        <v>546</v>
       </c>
       <c r="D112" s="3">
-        <v>16000</v>
-      </c>
-      <c r="E112" s="8" t="s">
+        <v>20500</v>
+      </c>
+      <c r="E112" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2398,15 +2416,15 @@
         <v>2</v>
       </c>
       <c r="B113" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C113" s="6">
-        <v>546</v>
+        <v>422</v>
       </c>
       <c r="D113" s="3">
-        <v>20000</v>
-      </c>
-      <c r="E113" s="8" t="s">
+        <v>39000</v>
+      </c>
+      <c r="E113" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2415,15 +2433,15 @@
         <v>2</v>
       </c>
       <c r="B114" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C114" s="6">
-        <v>422</v>
+        <v>1281</v>
       </c>
       <c r="D114" s="3">
-        <v>20000</v>
-      </c>
-      <c r="E114" s="8" t="s">
+        <v>39000</v>
+      </c>
+      <c r="E114" s="5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2432,13 +2450,13 @@
         <v>2</v>
       </c>
       <c r="B115" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C115" s="6">
-        <v>1281</v>
+        <v>2220</v>
       </c>
       <c r="D115" s="3">
-        <v>20000</v>
+        <v>34000</v>
       </c>
       <c r="E115" s="8" t="s">
         <v>1</v>
@@ -2449,13 +2467,13 @@
         <v>2</v>
       </c>
       <c r="B116" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C116" s="6">
-        <v>2220</v>
+        <v>2571</v>
       </c>
       <c r="D116" s="3">
-        <v>14000</v>
+        <v>34000</v>
       </c>
       <c r="E116" s="8" t="s">
         <v>1</v>
@@ -2463,33 +2481,33 @@
     </row>
     <row r="117" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B117" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C117" s="6">
-        <v>2571</v>
+        <v>2845</v>
       </c>
       <c r="D117" s="3">
-        <v>18000</v>
+        <v>10000</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" s="5">
         <v>3</v>
       </c>
-      <c r="B118" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C118" s="7">
-        <v>2845</v>
-      </c>
-      <c r="D118" s="4">
-        <v>7000</v>
+      <c r="B118" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C118" s="17">
+        <v>691</v>
+      </c>
+      <c r="D118" s="19">
+        <v>21000</v>
       </c>
       <c r="E118" s="8" t="s">
         <v>2</v>
@@ -2499,14 +2517,14 @@
       <c r="A119" s="5">
         <v>3</v>
       </c>
-      <c r="B119" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C119" s="7">
-        <v>691</v>
-      </c>
-      <c r="D119" s="4">
-        <v>20000</v>
+      <c r="B119" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C119" s="17">
+        <v>1533</v>
+      </c>
+      <c r="D119" s="19">
+        <v>26000</v>
       </c>
       <c r="E119" s="8" t="s">
         <v>2</v>
@@ -2516,14 +2534,14 @@
       <c r="A120" s="5">
         <v>3</v>
       </c>
-      <c r="B120" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C120" s="7">
-        <v>1533</v>
-      </c>
-      <c r="D120" s="4">
-        <v>22000</v>
+      <c r="B120" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C120" s="17">
+        <v>738</v>
+      </c>
+      <c r="D120" s="19">
+        <v>18000</v>
       </c>
       <c r="E120" s="8" t="s">
         <v>2</v>
@@ -2533,14 +2551,14 @@
       <c r="A121" s="5">
         <v>3</v>
       </c>
-      <c r="B121" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C121" s="7">
-        <v>738</v>
-      </c>
-      <c r="D121" s="4">
-        <v>20000</v>
+      <c r="B121" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C121" s="17">
+        <v>213</v>
+      </c>
+      <c r="D121" s="19">
+        <v>60000</v>
       </c>
       <c r="E121" s="8" t="s">
         <v>2</v>
@@ -2550,14 +2568,14 @@
       <c r="A122" s="5">
         <v>3</v>
       </c>
-      <c r="B122" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C122" s="7">
-        <v>213</v>
-      </c>
-      <c r="D122" s="4">
-        <v>13000</v>
+      <c r="B122" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C122" s="17">
+        <v>3009</v>
+      </c>
+      <c r="D122" s="19">
+        <v>35000</v>
       </c>
       <c r="E122" s="8" t="s">
         <v>2</v>
@@ -2565,33 +2583,33 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" s="5">
-        <v>3</v>
-      </c>
-      <c r="B123" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C123" s="7">
-        <v>3009</v>
-      </c>
-      <c r="D123" s="4">
-        <v>18000</v>
+        <v>4</v>
+      </c>
+      <c r="B123" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C123" s="17">
+        <v>3449</v>
+      </c>
+      <c r="D123" s="19">
+        <v>52000</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" s="5">
         <v>4</v>
       </c>
-      <c r="B124" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C124" s="7">
-        <v>3449</v>
-      </c>
-      <c r="D124" s="4">
-        <v>45000</v>
+      <c r="B124" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C124" s="17">
+        <v>1953</v>
+      </c>
+      <c r="D124" s="19">
+        <v>42000</v>
       </c>
       <c r="E124" s="8" t="s">
         <v>1</v>
@@ -2601,14 +2619,14 @@
       <c r="A125" s="5">
         <v>4</v>
       </c>
-      <c r="B125" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C125" s="7">
-        <v>1953</v>
-      </c>
-      <c r="D125" s="4">
-        <v>45000</v>
+      <c r="B125" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C125" s="17">
+        <v>2853</v>
+      </c>
+      <c r="D125" s="19">
+        <v>52000</v>
       </c>
       <c r="E125" s="8" t="s">
         <v>1</v>
@@ -2616,16 +2634,16 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="5">
-        <v>4</v>
-      </c>
-      <c r="B126" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C126" s="7">
-        <v>2853</v>
-      </c>
-      <c r="D126" s="4">
-        <v>40000</v>
+        <v>5</v>
+      </c>
+      <c r="B126" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C126" s="17">
+        <v>977</v>
+      </c>
+      <c r="D126" s="19">
+        <v>22500</v>
       </c>
       <c r="E126" s="8" t="s">
         <v>1</v>
@@ -2635,14 +2653,14 @@
       <c r="A127" s="5">
         <v>5</v>
       </c>
-      <c r="B127" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C127" s="7">
-        <v>977</v>
-      </c>
-      <c r="D127" s="4">
-        <v>18000</v>
+      <c r="B127" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C127" s="17">
+        <v>423</v>
+      </c>
+      <c r="D127" s="19">
+        <v>20500</v>
       </c>
       <c r="E127" s="8" t="s">
         <v>1</v>
@@ -2652,14 +2670,14 @@
       <c r="A128" s="5">
         <v>5</v>
       </c>
-      <c r="B128" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C128" s="7">
-        <v>423</v>
-      </c>
-      <c r="D128" s="4">
-        <v>16000</v>
+      <c r="B128" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C128" s="17">
+        <v>672</v>
+      </c>
+      <c r="D128" s="19">
+        <v>18000</v>
       </c>
       <c r="E128" s="8" t="s">
         <v>1</v>
@@ -2669,14 +2687,14 @@
       <c r="A129" s="5">
         <v>5</v>
       </c>
-      <c r="B129" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C129" s="7">
-        <v>672</v>
-      </c>
-      <c r="D129" s="4">
-        <v>18000</v>
+      <c r="B129" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C129" s="17">
+        <v>1929</v>
+      </c>
+      <c r="D129" s="19">
+        <v>17000</v>
       </c>
       <c r="E129" s="8" t="s">
         <v>1</v>
@@ -2686,14 +2704,14 @@
       <c r="A130" s="5">
         <v>5</v>
       </c>
-      <c r="B130" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C130" s="7">
-        <v>1929</v>
-      </c>
-      <c r="D130" s="4">
-        <v>14000</v>
+      <c r="B130" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C130" s="17">
+        <v>1087</v>
+      </c>
+      <c r="D130" s="19">
+        <v>20500</v>
       </c>
       <c r="E130" s="8" t="s">
         <v>1</v>
@@ -2703,14 +2721,14 @@
       <c r="A131" s="5">
         <v>5</v>
       </c>
-      <c r="B131" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C131" s="7">
-        <v>1087</v>
-      </c>
-      <c r="D131" s="4">
-        <v>16000</v>
+      <c r="B131" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C131" s="17">
+        <v>3179</v>
+      </c>
+      <c r="D131" s="19">
+        <v>16500</v>
       </c>
       <c r="E131" s="8" t="s">
         <v>1</v>
@@ -2718,16 +2736,16 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="5">
-        <v>5</v>
-      </c>
-      <c r="B132" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C132" s="7">
-        <v>3179</v>
-      </c>
-      <c r="D132" s="4">
-        <v>14000</v>
+        <v>6</v>
+      </c>
+      <c r="B132" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C132" s="17">
+        <v>1954</v>
+      </c>
+      <c r="D132" s="19">
+        <v>84000</v>
       </c>
       <c r="E132" s="8" t="s">
         <v>1</v>
@@ -2737,14 +2755,14 @@
       <c r="A133" s="5">
         <v>6</v>
       </c>
-      <c r="B133" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C133" s="7">
-        <v>1954</v>
-      </c>
-      <c r="D133" s="4">
-        <v>35000</v>
+      <c r="B133" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C133" s="17">
+        <v>1312</v>
+      </c>
+      <c r="D133" s="19">
+        <v>47000</v>
       </c>
       <c r="E133" s="8" t="s">
         <v>1</v>
@@ -2754,14 +2772,14 @@
       <c r="A134" s="5">
         <v>6</v>
       </c>
-      <c r="B134" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C134" s="7">
-        <v>1312</v>
-      </c>
-      <c r="D134" s="4">
-        <v>40000</v>
+      <c r="B134" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C134" s="17">
+        <v>874</v>
+      </c>
+      <c r="D134" s="19">
+        <v>94000</v>
       </c>
       <c r="E134" s="8" t="s">
         <v>1</v>
@@ -2769,33 +2787,33 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="5">
-        <v>6</v>
-      </c>
-      <c r="B135" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C135" s="7">
-        <v>874</v>
-      </c>
-      <c r="D135" s="4">
-        <v>40000</v>
+        <v>7</v>
+      </c>
+      <c r="B135" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C135" s="17">
+        <v>1899</v>
+      </c>
+      <c r="D135" s="19">
+        <v>15000</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" s="5">
         <v>7</v>
       </c>
-      <c r="B136" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C136" s="7">
-        <v>1899</v>
-      </c>
-      <c r="D136" s="4">
-        <v>15000</v>
+      <c r="B136" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C136" s="17">
+        <v>2985</v>
+      </c>
+      <c r="D136" s="19">
+        <v>10000</v>
       </c>
       <c r="E136" s="8" t="s">
         <v>3</v>
@@ -2805,14 +2823,14 @@
       <c r="A137" s="5">
         <v>7</v>
       </c>
-      <c r="B137" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C137" s="7">
-        <v>2985</v>
-      </c>
-      <c r="D137" s="4">
-        <v>10000</v>
+      <c r="B137" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C137" s="17">
+        <v>2184</v>
+      </c>
+      <c r="D137" s="19">
+        <v>15000</v>
       </c>
       <c r="E137" s="8" t="s">
         <v>3</v>
@@ -2822,14 +2840,14 @@
       <c r="A138" s="5">
         <v>7</v>
       </c>
-      <c r="B138" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C138" s="7">
-        <v>2184</v>
-      </c>
-      <c r="D138" s="4">
-        <v>15000</v>
+      <c r="B138" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C138" s="17">
+        <v>519</v>
+      </c>
+      <c r="D138" s="19">
+        <v>20000</v>
       </c>
       <c r="E138" s="8" t="s">
         <v>3</v>
@@ -2839,14 +2857,14 @@
       <c r="A139" s="5">
         <v>7</v>
       </c>
-      <c r="B139" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C139" s="7">
-        <v>519</v>
-      </c>
-      <c r="D139" s="4">
-        <v>20000</v>
+      <c r="B139" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C139" s="17">
+        <v>2183</v>
+      </c>
+      <c r="D139" s="19">
+        <v>10000</v>
       </c>
       <c r="E139" s="8" t="s">
         <v>3</v>
@@ -2856,14 +2874,14 @@
       <c r="A140" s="5">
         <v>7</v>
       </c>
-      <c r="B140" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C140" s="7">
-        <v>2183</v>
-      </c>
-      <c r="D140" s="4">
-        <v>10000</v>
+      <c r="B140" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C140" s="17">
+        <v>1884</v>
+      </c>
+      <c r="D140" s="19">
+        <v>16000</v>
       </c>
       <c r="E140" s="8" t="s">
         <v>3</v>
@@ -2873,14 +2891,14 @@
       <c r="A141" s="5">
         <v>7</v>
       </c>
-      <c r="B141" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C141" s="7">
-        <v>1884</v>
-      </c>
-      <c r="D141" s="4">
-        <v>16000</v>
+      <c r="B141" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C141" s="17">
+        <v>2185</v>
+      </c>
+      <c r="D141" s="19">
+        <v>10000</v>
       </c>
       <c r="E141" s="8" t="s">
         <v>3</v>
@@ -2890,14 +2908,14 @@
       <c r="A142" s="5">
         <v>7</v>
       </c>
-      <c r="B142" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C142" s="7">
-        <v>2185</v>
-      </c>
-      <c r="D142" s="4">
-        <v>10000</v>
+      <c r="B142" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C142" s="17">
+        <v>1885</v>
+      </c>
+      <c r="D142" s="19">
+        <v>13000</v>
       </c>
       <c r="E142" s="8" t="s">
         <v>3</v>
@@ -2907,14 +2925,14 @@
       <c r="A143" s="5">
         <v>7</v>
       </c>
-      <c r="B143" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C143" s="7">
-        <v>1885</v>
-      </c>
-      <c r="D143" s="4">
-        <v>13000</v>
+      <c r="B143" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C143" s="17">
+        <v>3389</v>
+      </c>
+      <c r="D143" s="19">
+        <v>8000</v>
       </c>
       <c r="E143" s="8" t="s">
         <v>3</v>
@@ -2924,14 +2942,14 @@
       <c r="A144" s="5">
         <v>7</v>
       </c>
-      <c r="B144" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C144" s="7">
-        <v>3389</v>
-      </c>
-      <c r="D144" s="4">
-        <v>8000</v>
+      <c r="B144" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C144" s="17">
+        <v>1883</v>
+      </c>
+      <c r="D144" s="19">
+        <v>16000</v>
       </c>
       <c r="E144" s="8" t="s">
         <v>3</v>
@@ -2939,33 +2957,33 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="5">
-        <v>7</v>
-      </c>
-      <c r="B145" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C145" s="7">
-        <v>1883</v>
-      </c>
-      <c r="D145" s="4">
-        <v>12000</v>
+        <v>9</v>
+      </c>
+      <c r="B145" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C145" s="17">
+        <v>2476</v>
+      </c>
+      <c r="D145" s="19">
+        <v>1490</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" s="5">
         <v>9</v>
       </c>
-      <c r="B146" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C146" s="7">
-        <v>2476</v>
-      </c>
-      <c r="D146" s="4">
-        <v>1490</v>
+      <c r="B146" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C146" s="17">
+        <v>2494</v>
+      </c>
+      <c r="D146" s="19">
+        <v>1412</v>
       </c>
       <c r="E146" s="8" t="s">
         <v>4</v>
@@ -2975,14 +2993,14 @@
       <c r="A147" s="5">
         <v>9</v>
       </c>
-      <c r="B147" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C147" s="7">
-        <v>2494</v>
-      </c>
-      <c r="D147" s="4">
-        <v>1412</v>
+      <c r="B147" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C147" s="17">
+        <v>2661</v>
+      </c>
+      <c r="D147" s="19">
+        <v>1257</v>
       </c>
       <c r="E147" s="8" t="s">
         <v>4</v>
@@ -2992,14 +3010,14 @@
       <c r="A148" s="5">
         <v>9</v>
       </c>
-      <c r="B148" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C148" s="7">
-        <v>2661</v>
-      </c>
-      <c r="D148" s="4">
-        <v>1257</v>
+      <c r="B148" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C148" s="17">
+        <v>3465</v>
+      </c>
+      <c r="D148" s="19">
+        <v>714</v>
       </c>
       <c r="E148" s="8" t="s">
         <v>4</v>
@@ -3009,13 +3027,13 @@
       <c r="A149" s="5">
         <v>9</v>
       </c>
-      <c r="B149" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C149" s="7">
-        <v>3465</v>
-      </c>
-      <c r="D149" s="4">
+      <c r="B149" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C149" s="17">
+        <v>1133</v>
+      </c>
+      <c r="D149" s="19">
         <v>714</v>
       </c>
       <c r="E149" s="8" t="s">
@@ -3026,13 +3044,13 @@
       <c r="A150" s="5">
         <v>9</v>
       </c>
-      <c r="B150" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C150" s="7">
-        <v>1133</v>
-      </c>
-      <c r="D150" s="4">
+      <c r="B150" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C150" s="17">
+        <v>3467</v>
+      </c>
+      <c r="D150" s="19">
         <v>714</v>
       </c>
       <c r="E150" s="8" t="s">
@@ -3041,16 +3059,16 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="5">
-        <v>9</v>
-      </c>
-      <c r="B151" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C151" s="7">
-        <v>3467</v>
-      </c>
-      <c r="D151" s="4">
-        <v>714</v>
+        <v>8</v>
+      </c>
+      <c r="B151" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C151" s="17">
+        <v>1762</v>
+      </c>
+      <c r="D151" s="19">
+        <v>42853</v>
       </c>
       <c r="E151" s="8" t="s">
         <v>4</v>
@@ -3060,14 +3078,14 @@
       <c r="A152" s="5">
         <v>8</v>
       </c>
-      <c r="B152" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C152" s="7">
-        <v>1762</v>
-      </c>
-      <c r="D152" s="4">
-        <v>42853</v>
+      <c r="B152" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C152" s="17">
+        <v>1778</v>
+      </c>
+      <c r="D152" s="19">
+        <v>33671</v>
       </c>
       <c r="E152" s="8" t="s">
         <v>4</v>
@@ -3077,14 +3095,14 @@
       <c r="A153" s="5">
         <v>8</v>
       </c>
-      <c r="B153" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C153" s="7">
-        <v>1778</v>
-      </c>
-      <c r="D153" s="4">
-        <v>40707</v>
+      <c r="B153" s="15">
+        <v>46235</v>
+      </c>
+      <c r="C153" s="17">
+        <v>2727</v>
+      </c>
+      <c r="D153" s="19">
+        <v>29079</v>
       </c>
       <c r="E153" s="8" t="s">
         <v>4</v>
@@ -3092,18 +3110,868 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="5">
+        <v>1</v>
+      </c>
+      <c r="B154" s="15">
+        <v>46266</v>
+      </c>
+      <c r="C154" s="17">
+        <v>27</v>
+      </c>
+      <c r="D154" s="19">
+        <v>310000</v>
+      </c>
+      <c r="E154" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A155" s="5">
+        <v>1</v>
+      </c>
+      <c r="B155" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C155" s="7">
+        <v>1139</v>
+      </c>
+      <c r="D155" s="4">
+        <v>320000</v>
+      </c>
+      <c r="E155" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A156" s="5">
+        <v>1</v>
+      </c>
+      <c r="B156" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C156" s="7">
+        <v>675</v>
+      </c>
+      <c r="D156" s="4">
+        <v>210000</v>
+      </c>
+      <c r="E156" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A157" s="5">
+        <v>1</v>
+      </c>
+      <c r="B157" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C157" s="7">
+        <v>58</v>
+      </c>
+      <c r="D157" s="4">
+        <v>170000</v>
+      </c>
+      <c r="E157" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A158" s="5">
+        <v>1</v>
+      </c>
+      <c r="B158" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C158" s="7">
+        <v>841</v>
+      </c>
+      <c r="D158" s="4">
+        <v>100000</v>
+      </c>
+      <c r="E158" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A159" s="5">
+        <v>1</v>
+      </c>
+      <c r="B159" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C159" s="7">
+        <v>13148</v>
+      </c>
+      <c r="D159" s="4">
+        <v>150000</v>
+      </c>
+      <c r="E159" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A160" s="5">
+        <v>1</v>
+      </c>
+      <c r="B160" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C160" s="7">
+        <v>805</v>
+      </c>
+      <c r="D160" s="4">
+        <v>300000</v>
+      </c>
+      <c r="E160" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A161" s="5">
+        <v>1</v>
+      </c>
+      <c r="B161" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C161" s="7">
+        <v>3403</v>
+      </c>
+      <c r="D161" s="4">
+        <v>250000</v>
+      </c>
+      <c r="E161" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A162" s="5">
+        <v>2</v>
+      </c>
+      <c r="B162" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C162" s="7">
+        <v>1898</v>
+      </c>
+      <c r="D162" s="4">
+        <v>250000</v>
+      </c>
+      <c r="E162" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A163" s="5">
+        <v>2</v>
+      </c>
+      <c r="B163" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C163" s="7">
+        <v>546</v>
+      </c>
+      <c r="D163" s="4">
+        <v>260000</v>
+      </c>
+      <c r="E163" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A164" s="5">
+        <v>2</v>
+      </c>
+      <c r="B164" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C164" s="7">
+        <v>422</v>
+      </c>
+      <c r="D164" s="4">
+        <v>260000</v>
+      </c>
+      <c r="E164" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A165" s="5">
+        <v>2</v>
+      </c>
+      <c r="B165" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C165" s="7">
+        <v>1281</v>
+      </c>
+      <c r="D165" s="4">
+        <v>280000</v>
+      </c>
+      <c r="E165" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A166" s="5">
+        <v>2</v>
+      </c>
+      <c r="B166" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C166" s="7">
+        <v>2220</v>
+      </c>
+      <c r="D166" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E166" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A167" s="5">
+        <v>2</v>
+      </c>
+      <c r="B167" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C167" s="7">
+        <v>2571</v>
+      </c>
+      <c r="D167" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E167" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A168" s="5">
+        <v>3</v>
+      </c>
+      <c r="B168" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C168" s="7">
+        <v>2845</v>
+      </c>
+      <c r="D168" s="4">
+        <v>100000</v>
+      </c>
+      <c r="E168" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A169" s="5">
+        <v>3</v>
+      </c>
+      <c r="B169" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C169" s="7">
+        <v>691</v>
+      </c>
+      <c r="D169" s="4">
+        <v>250000</v>
+      </c>
+      <c r="E169" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A170" s="5">
+        <v>3</v>
+      </c>
+      <c r="B170" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C170" s="7">
+        <v>1533</v>
+      </c>
+      <c r="D170" s="4">
+        <v>340000</v>
+      </c>
+      <c r="E170" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A171" s="5">
+        <v>3</v>
+      </c>
+      <c r="B171" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C171" s="7">
+        <v>738</v>
+      </c>
+      <c r="D171" s="4">
+        <v>220000</v>
+      </c>
+      <c r="E171" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A172" s="5">
+        <v>3</v>
+      </c>
+      <c r="B172" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C172" s="7">
+        <v>213</v>
+      </c>
+      <c r="D172" s="4">
+        <v>80000</v>
+      </c>
+      <c r="E172" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A173" s="5">
+        <v>3</v>
+      </c>
+      <c r="B173" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C173" s="7">
+        <v>3009</v>
+      </c>
+      <c r="D173" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E173" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A174" s="5">
+        <v>4</v>
+      </c>
+      <c r="B174" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C174" s="7">
+        <v>3449</v>
+      </c>
+      <c r="D174" s="4">
+        <v>230000</v>
+      </c>
+      <c r="E174" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A175" s="5">
+        <v>4</v>
+      </c>
+      <c r="B175" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C175" s="7">
+        <v>1953</v>
+      </c>
+      <c r="D175" s="4">
+        <v>220000</v>
+      </c>
+      <c r="E175" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A176" s="5">
+        <v>4</v>
+      </c>
+      <c r="B176" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C176" s="7">
+        <v>2853</v>
+      </c>
+      <c r="D176" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E176" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A177" s="5">
+        <v>5</v>
+      </c>
+      <c r="B177" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C177" s="7">
+        <v>977</v>
+      </c>
+      <c r="D177" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E177" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A178" s="5">
+        <v>5</v>
+      </c>
+      <c r="B178" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C178" s="7">
+        <v>423</v>
+      </c>
+      <c r="D178" s="4">
+        <v>250000</v>
+      </c>
+      <c r="E178" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A179" s="5">
+        <v>5</v>
+      </c>
+      <c r="B179" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C179" s="7">
+        <v>672</v>
+      </c>
+      <c r="D179" s="4">
+        <v>250000</v>
+      </c>
+      <c r="E179" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A180" s="5">
+        <v>5</v>
+      </c>
+      <c r="B180" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C180" s="7">
+        <v>1929</v>
+      </c>
+      <c r="D180" s="4">
+        <v>210000</v>
+      </c>
+      <c r="E180" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A181" s="5">
+        <v>5</v>
+      </c>
+      <c r="B181" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C181" s="7">
+        <v>1087</v>
+      </c>
+      <c r="D181" s="4">
+        <v>170000</v>
+      </c>
+      <c r="E181" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A182" s="5">
+        <v>5</v>
+      </c>
+      <c r="B182" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C182" s="7">
+        <v>3179</v>
+      </c>
+      <c r="D182" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A183" s="5">
+        <v>6</v>
+      </c>
+      <c r="B183" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C183" s="7">
+        <v>1954</v>
+      </c>
+      <c r="D183" s="4">
+        <v>180000</v>
+      </c>
+      <c r="E183" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A184" s="5">
+        <v>6</v>
+      </c>
+      <c r="B184" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C184" s="7">
+        <v>1312</v>
+      </c>
+      <c r="D184" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E184" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A185" s="5">
+        <v>6</v>
+      </c>
+      <c r="B185" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C185" s="7">
+        <v>874</v>
+      </c>
+      <c r="D185" s="4">
+        <v>200000</v>
+      </c>
+      <c r="E185" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A186" s="5">
+        <v>7</v>
+      </c>
+      <c r="B186" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C186" s="7">
+        <v>1899</v>
+      </c>
+      <c r="D186" s="4">
+        <v>245000</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A187" s="5">
+        <v>7</v>
+      </c>
+      <c r="B187" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C187" s="7">
+        <v>2985</v>
+      </c>
+      <c r="D187" s="4">
+        <v>126000</v>
+      </c>
+      <c r="E187" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A188" s="5">
+        <v>7</v>
+      </c>
+      <c r="B188" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C188" s="7">
+        <v>2184</v>
+      </c>
+      <c r="D188" s="4">
+        <v>195000</v>
+      </c>
+      <c r="E188" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A189" s="5">
+        <v>7</v>
+      </c>
+      <c r="B189" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C189" s="7">
+        <v>519</v>
+      </c>
+      <c r="D189" s="4">
+        <v>360000</v>
+      </c>
+      <c r="E189" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A190" s="5">
+        <v>7</v>
+      </c>
+      <c r="B190" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C190" s="7">
+        <v>2183</v>
+      </c>
+      <c r="D190" s="4">
+        <v>136000</v>
+      </c>
+      <c r="E190" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A191" s="5">
+        <v>7</v>
+      </c>
+      <c r="B191" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C191" s="7">
+        <v>1884</v>
+      </c>
+      <c r="D191" s="4">
+        <v>195000</v>
+      </c>
+      <c r="E191" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A192" s="5">
+        <v>7</v>
+      </c>
+      <c r="B192" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C192" s="7">
+        <v>2185</v>
+      </c>
+      <c r="D192" s="4">
+        <v>136000</v>
+      </c>
+      <c r="E192" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A193" s="5">
+        <v>7</v>
+      </c>
+      <c r="B193" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C193" s="7">
+        <v>1885</v>
+      </c>
+      <c r="D193" s="4">
+        <v>160000</v>
+      </c>
+      <c r="E193" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A194" s="5">
+        <v>7</v>
+      </c>
+      <c r="B194" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C194" s="7">
+        <v>3389</v>
+      </c>
+      <c r="D194" s="4">
+        <v>96000</v>
+      </c>
+      <c r="E194" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A195" s="5">
+        <v>7</v>
+      </c>
+      <c r="B195" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C195" s="7">
+        <v>1883</v>
+      </c>
+      <c r="D195" s="4">
+        <v>210000</v>
+      </c>
+      <c r="E195" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A196" s="5">
+        <v>9</v>
+      </c>
+      <c r="B196" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C196" s="7">
+        <v>2476</v>
+      </c>
+      <c r="D196" s="4">
+        <v>190000</v>
+      </c>
+      <c r="E196" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A197" s="5">
+        <v>9</v>
+      </c>
+      <c r="B197" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C197" s="7">
+        <v>2494</v>
+      </c>
+      <c r="D197" s="4">
+        <v>150000</v>
+      </c>
+      <c r="E197" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A198" s="5">
+        <v>9</v>
+      </c>
+      <c r="B198" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C198" s="7">
+        <v>2661</v>
+      </c>
+      <c r="D198" s="4">
+        <v>125000</v>
+      </c>
+      <c r="E198" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A199" s="5">
+        <v>9</v>
+      </c>
+      <c r="B199" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C199" s="7">
+        <v>3465</v>
+      </c>
+      <c r="D199" s="4">
+        <v>115667</v>
+      </c>
+      <c r="E199" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A200" s="5">
+        <v>9</v>
+      </c>
+      <c r="B200" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C200" s="7">
+        <v>1133</v>
+      </c>
+      <c r="D200" s="4">
+        <v>115667</v>
+      </c>
+      <c r="E200" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A201" s="5">
+        <v>9</v>
+      </c>
+      <c r="B201" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C201" s="7">
+        <v>3467</v>
+      </c>
+      <c r="D201" s="4">
+        <v>115667</v>
+      </c>
+      <c r="E201" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A202" s="5">
         <v>8</v>
       </c>
-      <c r="B154" s="2">
-        <v>46204</v>
-      </c>
-      <c r="C154" s="7">
+      <c r="B202" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C202" s="7">
+        <v>1762</v>
+      </c>
+      <c r="D202" s="4">
+        <v>280000</v>
+      </c>
+      <c r="E202" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A203" s="5">
+        <v>8</v>
+      </c>
+      <c r="B203" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C203" s="7">
+        <v>1778</v>
+      </c>
+      <c r="D203" s="4">
+        <v>265978</v>
+      </c>
+      <c r="E203" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A204" s="5">
+        <v>8</v>
+      </c>
+      <c r="B204" s="2">
+        <v>46266</v>
+      </c>
+      <c r="C204" s="7">
         <v>2727</v>
       </c>
-      <c r="D154" s="4">
-        <v>39634</v>
-      </c>
-      <c r="E154" s="8" t="s">
+      <c r="D204" s="4">
+        <v>190000</v>
+      </c>
+      <c r="E204" s="8" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ajuste meta mes 9
</commit_message>
<xml_diff>
--- a/data/meta_marcas_televendas.xlsx
+++ b/data/meta_marcas_televendas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153EB97A-1B1A-4F81-AA16-43F2FC9D9A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB70181-1B61-4883-94AE-5F5504672840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="9">
   <si>
     <t>DATA</t>
   </si>
@@ -496,7 +496,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="5"/>
@@ -1396,13 +1396,13 @@
         <v>1</v>
       </c>
       <c r="B53" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C53" s="6">
-        <v>1139</v>
+        <v>27</v>
       </c>
       <c r="D53" s="3">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="E53" s="8" t="s">
         <v>2</v>
@@ -1413,13 +1413,13 @@
         <v>1</v>
       </c>
       <c r="B54" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C54" s="6">
-        <v>675</v>
+        <v>1139</v>
       </c>
       <c r="D54" s="3">
-        <v>7000</v>
+        <v>30000</v>
       </c>
       <c r="E54" s="8" t="s">
         <v>2</v>
@@ -1430,10 +1430,10 @@
         <v>1</v>
       </c>
       <c r="B55" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C55" s="6">
-        <v>58</v>
+        <v>675</v>
       </c>
       <c r="D55" s="3">
         <v>7000</v>
@@ -1447,10 +1447,10 @@
         <v>1</v>
       </c>
       <c r="B56" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C56" s="6">
-        <v>841</v>
+        <v>58</v>
       </c>
       <c r="D56" s="3">
         <v>7000</v>
@@ -1464,10 +1464,10 @@
         <v>1</v>
       </c>
       <c r="B57" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C57" s="6">
-        <v>13148</v>
+        <v>841</v>
       </c>
       <c r="D57" s="3">
         <v>7000</v>
@@ -1481,13 +1481,13 @@
         <v>1</v>
       </c>
       <c r="B58" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C58" s="6">
-        <v>805</v>
+        <v>13148</v>
       </c>
       <c r="D58" s="3">
-        <v>17000</v>
+        <v>7000</v>
       </c>
       <c r="E58" s="8" t="s">
         <v>2</v>
@@ -1498,13 +1498,13 @@
         <v>1</v>
       </c>
       <c r="B59" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C59" s="6">
-        <v>3403</v>
+        <v>805</v>
       </c>
       <c r="D59" s="3">
-        <v>10000</v>
+        <v>21000</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>2</v>
@@ -1512,19 +1512,19 @@
     </row>
     <row r="60" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B60" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C60" s="6">
-        <v>1898</v>
+        <v>3403</v>
       </c>
       <c r="D60" s="3">
-        <v>16000</v>
+        <v>13000</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1532,13 +1532,13 @@
         <v>2</v>
       </c>
       <c r="B61" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C61" s="6">
-        <v>546</v>
+        <v>1898</v>
       </c>
       <c r="D61" s="3">
-        <v>20000</v>
+        <v>37500</v>
       </c>
       <c r="E61" s="8" t="s">
         <v>1</v>
@@ -1549,13 +1549,13 @@
         <v>2</v>
       </c>
       <c r="B62" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C62" s="6">
-        <v>422</v>
+        <v>546</v>
       </c>
       <c r="D62" s="3">
-        <v>20000</v>
+        <v>20500</v>
       </c>
       <c r="E62" s="8" t="s">
         <v>1</v>
@@ -1566,13 +1566,13 @@
         <v>2</v>
       </c>
       <c r="B63" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C63" s="6">
-        <v>1281</v>
+        <v>422</v>
       </c>
       <c r="D63" s="3">
-        <v>20000</v>
+        <v>39000</v>
       </c>
       <c r="E63" s="8" t="s">
         <v>1</v>
@@ -1583,13 +1583,13 @@
         <v>2</v>
       </c>
       <c r="B64" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C64" s="6">
-        <v>2220</v>
+        <v>1281</v>
       </c>
       <c r="D64" s="3">
-        <v>14000</v>
+        <v>39000</v>
       </c>
       <c r="E64" s="8" t="s">
         <v>1</v>
@@ -1600,13 +1600,13 @@
         <v>2</v>
       </c>
       <c r="B65" s="1">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C65" s="6">
-        <v>2571</v>
+        <v>2220</v>
       </c>
       <c r="D65" s="3">
-        <v>18000</v>
+        <v>34000</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>1</v>
@@ -1614,19 +1614,19 @@
     </row>
     <row r="66" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B66" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C66" s="16">
-        <v>2845</v>
+        <v>2571</v>
       </c>
       <c r="D66" s="18">
-        <v>7000</v>
+        <v>34000</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1634,13 +1634,13 @@
         <v>3</v>
       </c>
       <c r="B67" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C67" s="16">
-        <v>691</v>
+        <v>2845</v>
       </c>
       <c r="D67" s="18">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="E67" s="8" t="s">
         <v>2</v>
@@ -1651,13 +1651,13 @@
         <v>3</v>
       </c>
       <c r="B68" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C68" s="16">
-        <v>1533</v>
+        <v>691</v>
       </c>
       <c r="D68" s="18">
-        <v>22000</v>
+        <v>21000</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>2</v>
@@ -1668,13 +1668,13 @@
         <v>3</v>
       </c>
       <c r="B69" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C69" s="16">
-        <v>738</v>
+        <v>1533</v>
       </c>
       <c r="D69" s="18">
-        <v>20000</v>
+        <v>26000</v>
       </c>
       <c r="E69" s="8" t="s">
         <v>2</v>
@@ -1685,13 +1685,13 @@
         <v>3</v>
       </c>
       <c r="B70" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C70" s="16">
-        <v>213</v>
+        <v>738</v>
       </c>
       <c r="D70" s="18">
-        <v>13000</v>
+        <v>18000</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>2</v>
@@ -1702,13 +1702,13 @@
         <v>3</v>
       </c>
       <c r="B71" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C71" s="16">
-        <v>3009</v>
+        <v>213</v>
       </c>
       <c r="D71" s="18">
-        <v>18000</v>
+        <v>60000</v>
       </c>
       <c r="E71" s="8" t="s">
         <v>2</v>
@@ -1716,19 +1716,19 @@
     </row>
     <row r="72" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B72" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C72" s="16">
-        <v>3449</v>
+        <v>3009</v>
       </c>
       <c r="D72" s="18">
-        <v>45000</v>
+        <v>35000</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1736,13 +1736,13 @@
         <v>4</v>
       </c>
       <c r="B73" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C73" s="16">
-        <v>1953</v>
+        <v>3449</v>
       </c>
       <c r="D73" s="18">
-        <v>45000</v>
+        <v>52000</v>
       </c>
       <c r="E73" s="8" t="s">
         <v>1</v>
@@ -1753,13 +1753,13 @@
         <v>4</v>
       </c>
       <c r="B74" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C74" s="16">
-        <v>2853</v>
+        <v>1953</v>
       </c>
       <c r="D74" s="18">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="E74" s="8" t="s">
         <v>1</v>
@@ -1767,16 +1767,16 @@
     </row>
     <row r="75" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B75" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C75" s="16">
-        <v>977</v>
+        <v>2853</v>
       </c>
       <c r="D75" s="18">
-        <v>18000</v>
+        <v>52000</v>
       </c>
       <c r="E75" s="8" t="s">
         <v>1</v>
@@ -1787,13 +1787,13 @@
         <v>5</v>
       </c>
       <c r="B76" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C76" s="16">
-        <v>423</v>
+        <v>977</v>
       </c>
       <c r="D76" s="18">
-        <v>16000</v>
+        <v>22500</v>
       </c>
       <c r="E76" s="8" t="s">
         <v>1</v>
@@ -1804,13 +1804,13 @@
         <v>5</v>
       </c>
       <c r="B77" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C77" s="16">
-        <v>672</v>
+        <v>423</v>
       </c>
       <c r="D77" s="18">
-        <v>18000</v>
+        <v>20500</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>1</v>
@@ -1821,13 +1821,13 @@
         <v>5</v>
       </c>
       <c r="B78" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C78" s="16">
-        <v>1929</v>
+        <v>672</v>
       </c>
       <c r="D78" s="18">
-        <v>14000</v>
+        <v>18000</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>1</v>
@@ -1838,13 +1838,13 @@
         <v>5</v>
       </c>
       <c r="B79" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C79" s="16">
-        <v>1087</v>
+        <v>1929</v>
       </c>
       <c r="D79" s="18">
-        <v>16000</v>
+        <v>17000</v>
       </c>
       <c r="E79" s="8" t="s">
         <v>1</v>
@@ -1855,13 +1855,13 @@
         <v>5</v>
       </c>
       <c r="B80" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C80" s="16">
-        <v>3179</v>
+        <v>1087</v>
       </c>
       <c r="D80" s="18">
-        <v>14000</v>
+        <v>20500</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>1</v>
@@ -1869,16 +1869,16 @@
     </row>
     <row r="81" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B81" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C81" s="16">
-        <v>1954</v>
+        <v>3179</v>
       </c>
       <c r="D81" s="18">
-        <v>35000</v>
+        <v>16500</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>1</v>
@@ -1889,13 +1889,13 @@
         <v>6</v>
       </c>
       <c r="B82" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C82" s="16">
-        <v>1312</v>
+        <v>1954</v>
       </c>
       <c r="D82" s="18">
-        <v>40000</v>
+        <v>84000</v>
       </c>
       <c r="E82" s="8" t="s">
         <v>1</v>
@@ -1906,13 +1906,13 @@
         <v>6</v>
       </c>
       <c r="B83" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C83" s="16">
-        <v>874</v>
+        <v>1312</v>
       </c>
       <c r="D83" s="18">
-        <v>40000</v>
+        <v>47000</v>
       </c>
       <c r="E83" s="8" t="s">
         <v>1</v>
@@ -1920,19 +1920,19 @@
     </row>
     <row r="84" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B84" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C84" s="16">
-        <v>1899</v>
+        <v>874</v>
       </c>
       <c r="D84" s="18">
-        <v>15000</v>
+        <v>94000</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1940,13 +1940,13 @@
         <v>7</v>
       </c>
       <c r="B85" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C85" s="16">
-        <v>2985</v>
+        <v>1899</v>
       </c>
       <c r="D85" s="18">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E85" s="8" t="s">
         <v>3</v>
@@ -1957,13 +1957,13 @@
         <v>7</v>
       </c>
       <c r="B86" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C86" s="16">
-        <v>2184</v>
+        <v>2985</v>
       </c>
       <c r="D86" s="18">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>3</v>
@@ -1974,13 +1974,13 @@
         <v>7</v>
       </c>
       <c r="B87" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C87" s="16">
-        <v>519</v>
+        <v>2184</v>
       </c>
       <c r="D87" s="18">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="E87" s="8" t="s">
         <v>3</v>
@@ -1991,13 +1991,13 @@
         <v>7</v>
       </c>
       <c r="B88" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C88" s="16">
-        <v>2183</v>
+        <v>519</v>
       </c>
       <c r="D88" s="18">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E88" s="8" t="s">
         <v>3</v>
@@ -2008,13 +2008,13 @@
         <v>7</v>
       </c>
       <c r="B89" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C89" s="16">
-        <v>1884</v>
+        <v>2183</v>
       </c>
       <c r="D89" s="18">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>3</v>
@@ -2025,13 +2025,13 @@
         <v>7</v>
       </c>
       <c r="B90" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C90" s="16">
-        <v>2185</v>
+        <v>1884</v>
       </c>
       <c r="D90" s="18">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="E90" s="8" t="s">
         <v>3</v>
@@ -2042,13 +2042,13 @@
         <v>7</v>
       </c>
       <c r="B91" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C91" s="16">
-        <v>1885</v>
+        <v>2185</v>
       </c>
       <c r="D91" s="18">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="E91" s="8" t="s">
         <v>3</v>
@@ -2059,13 +2059,13 @@
         <v>7</v>
       </c>
       <c r="B92" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C92" s="16">
-        <v>3389</v>
+        <v>1885</v>
       </c>
       <c r="D92" s="18">
-        <v>8000</v>
+        <v>13000</v>
       </c>
       <c r="E92" s="8" t="s">
         <v>3</v>
@@ -2076,13 +2076,13 @@
         <v>7</v>
       </c>
       <c r="B93" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C93" s="16">
-        <v>1883</v>
+        <v>3389</v>
       </c>
       <c r="D93" s="18">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="E93" s="8" t="s">
         <v>3</v>
@@ -2090,19 +2090,19 @@
     </row>
     <row r="94" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B94" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C94" s="16">
-        <v>2476</v>
+        <v>1883</v>
       </c>
       <c r="D94" s="18">
-        <v>1490</v>
+        <v>16000</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2110,13 +2110,13 @@
         <v>9</v>
       </c>
       <c r="B95" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C95" s="16">
-        <v>2494</v>
+        <v>2476</v>
       </c>
       <c r="D95" s="18">
-        <v>1412</v>
+        <v>1490</v>
       </c>
       <c r="E95" s="8" t="s">
         <v>4</v>
@@ -2127,13 +2127,13 @@
         <v>9</v>
       </c>
       <c r="B96" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C96" s="16">
-        <v>2661</v>
+        <v>2494</v>
       </c>
       <c r="D96" s="18">
-        <v>1257</v>
+        <v>1412</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>4</v>
@@ -2144,13 +2144,13 @@
         <v>9</v>
       </c>
       <c r="B97" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C97" s="16">
-        <v>3465</v>
+        <v>2661</v>
       </c>
       <c r="D97" s="18">
-        <v>714</v>
+        <v>1257</v>
       </c>
       <c r="E97" s="8" t="s">
         <v>4</v>
@@ -2161,10 +2161,10 @@
         <v>9</v>
       </c>
       <c r="B98" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C98" s="16">
-        <v>1133</v>
+        <v>3465</v>
       </c>
       <c r="D98" s="18">
         <v>714</v>
@@ -2178,10 +2178,10 @@
         <v>9</v>
       </c>
       <c r="B99" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C99" s="16">
-        <v>3467</v>
+        <v>1133</v>
       </c>
       <c r="D99" s="18">
         <v>714</v>
@@ -2192,16 +2192,16 @@
     </row>
     <row r="100" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B100" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C100" s="16">
-        <v>1762</v>
+        <v>3467</v>
       </c>
       <c r="D100" s="18">
-        <v>42853</v>
+        <v>714</v>
       </c>
       <c r="E100" s="8" t="s">
         <v>4</v>
@@ -2212,13 +2212,13 @@
         <v>8</v>
       </c>
       <c r="B101" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C101" s="16">
-        <v>1778</v>
+        <v>1762</v>
       </c>
       <c r="D101" s="18">
-        <v>40707</v>
+        <v>42853</v>
       </c>
       <c r="E101" s="8" t="s">
         <v>4</v>
@@ -2229,13 +2229,13 @@
         <v>8</v>
       </c>
       <c r="B102" s="14">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="C102" s="16">
-        <v>2727</v>
+        <v>1778</v>
       </c>
       <c r="D102" s="18">
-        <v>39634</v>
+        <v>33671</v>
       </c>
       <c r="E102" s="8" t="s">
         <v>4</v>
@@ -2243,19 +2243,19 @@
     </row>
     <row r="103" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B103" s="1">
         <v>46235</v>
       </c>
       <c r="C103" s="6">
-        <v>27</v>
+        <v>2727</v>
       </c>
       <c r="D103" s="3">
-        <v>15000</v>
+        <v>29079</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2263,13 +2263,13 @@
         <v>1</v>
       </c>
       <c r="B104" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C104" s="6">
-        <v>1139</v>
+        <v>27</v>
       </c>
       <c r="D104" s="3">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>2</v>
@@ -2280,13 +2280,13 @@
         <v>1</v>
       </c>
       <c r="B105" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C105" s="6">
-        <v>675</v>
+        <v>1139</v>
       </c>
       <c r="D105" s="3">
-        <v>7000</v>
+        <v>30000</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>2</v>
@@ -2297,10 +2297,10 @@
         <v>1</v>
       </c>
       <c r="B106" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C106" s="6">
-        <v>58</v>
+        <v>675</v>
       </c>
       <c r="D106" s="3">
         <v>7000</v>
@@ -2314,10 +2314,10 @@
         <v>1</v>
       </c>
       <c r="B107" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C107" s="6">
-        <v>841</v>
+        <v>58</v>
       </c>
       <c r="D107" s="3">
         <v>7000</v>
@@ -2331,10 +2331,10 @@
         <v>1</v>
       </c>
       <c r="B108" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C108" s="6">
-        <v>13148</v>
+        <v>841</v>
       </c>
       <c r="D108" s="3">
         <v>7000</v>
@@ -2348,13 +2348,13 @@
         <v>1</v>
       </c>
       <c r="B109" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C109" s="6">
-        <v>805</v>
+        <v>13148</v>
       </c>
       <c r="D109" s="3">
-        <v>21000</v>
+        <v>7000</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>2</v>
@@ -2365,13 +2365,13 @@
         <v>1</v>
       </c>
       <c r="B110" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C110" s="6">
-        <v>3403</v>
+        <v>805</v>
       </c>
       <c r="D110" s="3">
-        <v>13000</v>
+        <v>17000</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>2</v>
@@ -2379,19 +2379,19 @@
     </row>
     <row r="111" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B111" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C111" s="6">
-        <v>1898</v>
+        <v>3403</v>
       </c>
       <c r="D111" s="3">
-        <v>37500</v>
+        <v>10000</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2399,13 +2399,13 @@
         <v>2</v>
       </c>
       <c r="B112" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C112" s="6">
-        <v>546</v>
+        <v>1898</v>
       </c>
       <c r="D112" s="3">
-        <v>20500</v>
+        <v>16000</v>
       </c>
       <c r="E112" s="5" t="s">
         <v>1</v>
@@ -2416,13 +2416,13 @@
         <v>2</v>
       </c>
       <c r="B113" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C113" s="6">
-        <v>422</v>
+        <v>546</v>
       </c>
       <c r="D113" s="3">
-        <v>39000</v>
+        <v>20000</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>1</v>
@@ -2433,13 +2433,13 @@
         <v>2</v>
       </c>
       <c r="B114" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C114" s="6">
-        <v>1281</v>
+        <v>422</v>
       </c>
       <c r="D114" s="3">
-        <v>39000</v>
+        <v>20000</v>
       </c>
       <c r="E114" s="5" t="s">
         <v>1</v>
@@ -2450,13 +2450,13 @@
         <v>2</v>
       </c>
       <c r="B115" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C115" s="6">
-        <v>2220</v>
+        <v>1281</v>
       </c>
       <c r="D115" s="3">
-        <v>34000</v>
+        <v>20000</v>
       </c>
       <c r="E115" s="8" t="s">
         <v>1</v>
@@ -2467,13 +2467,13 @@
         <v>2</v>
       </c>
       <c r="B116" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C116" s="6">
-        <v>2571</v>
+        <v>2220</v>
       </c>
       <c r="D116" s="3">
-        <v>34000</v>
+        <v>14000</v>
       </c>
       <c r="E116" s="8" t="s">
         <v>1</v>
@@ -2481,19 +2481,19 @@
     </row>
     <row r="117" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B117" s="1">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C117" s="6">
-        <v>2845</v>
+        <v>2571</v>
       </c>
       <c r="D117" s="3">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.3">
@@ -2501,13 +2501,13 @@
         <v>3</v>
       </c>
       <c r="B118" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C118" s="17">
-        <v>691</v>
+        <v>2845</v>
       </c>
       <c r="D118" s="19">
-        <v>21000</v>
+        <v>7000</v>
       </c>
       <c r="E118" s="8" t="s">
         <v>2</v>
@@ -2518,13 +2518,13 @@
         <v>3</v>
       </c>
       <c r="B119" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C119" s="17">
-        <v>1533</v>
+        <v>691</v>
       </c>
       <c r="D119" s="19">
-        <v>26000</v>
+        <v>20000</v>
       </c>
       <c r="E119" s="8" t="s">
         <v>2</v>
@@ -2535,13 +2535,13 @@
         <v>3</v>
       </c>
       <c r="B120" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C120" s="17">
-        <v>738</v>
+        <v>1533</v>
       </c>
       <c r="D120" s="19">
-        <v>18000</v>
+        <v>22000</v>
       </c>
       <c r="E120" s="8" t="s">
         <v>2</v>
@@ -2552,13 +2552,13 @@
         <v>3</v>
       </c>
       <c r="B121" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C121" s="17">
-        <v>213</v>
+        <v>738</v>
       </c>
       <c r="D121" s="19">
-        <v>60000</v>
+        <v>20000</v>
       </c>
       <c r="E121" s="8" t="s">
         <v>2</v>
@@ -2569,13 +2569,13 @@
         <v>3</v>
       </c>
       <c r="B122" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C122" s="17">
-        <v>3009</v>
+        <v>213</v>
       </c>
       <c r="D122" s="19">
-        <v>35000</v>
+        <v>13000</v>
       </c>
       <c r="E122" s="8" t="s">
         <v>2</v>
@@ -2583,19 +2583,19 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B123" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C123" s="17">
-        <v>3449</v>
+        <v>3009</v>
       </c>
       <c r="D123" s="19">
-        <v>52000</v>
+        <v>18000</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.3">
@@ -2603,13 +2603,13 @@
         <v>4</v>
       </c>
       <c r="B124" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C124" s="17">
-        <v>1953</v>
+        <v>3449</v>
       </c>
       <c r="D124" s="19">
-        <v>42000</v>
+        <v>45000</v>
       </c>
       <c r="E124" s="8" t="s">
         <v>1</v>
@@ -2620,13 +2620,13 @@
         <v>4</v>
       </c>
       <c r="B125" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C125" s="17">
-        <v>2853</v>
+        <v>1953</v>
       </c>
       <c r="D125" s="19">
-        <v>52000</v>
+        <v>45000</v>
       </c>
       <c r="E125" s="8" t="s">
         <v>1</v>
@@ -2634,16 +2634,16 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B126" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C126" s="17">
-        <v>977</v>
+        <v>2853</v>
       </c>
       <c r="D126" s="19">
-        <v>22500</v>
+        <v>40000</v>
       </c>
       <c r="E126" s="8" t="s">
         <v>1</v>
@@ -2654,13 +2654,13 @@
         <v>5</v>
       </c>
       <c r="B127" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C127" s="17">
-        <v>423</v>
+        <v>977</v>
       </c>
       <c r="D127" s="19">
-        <v>20500</v>
+        <v>18000</v>
       </c>
       <c r="E127" s="8" t="s">
         <v>1</v>
@@ -2671,13 +2671,13 @@
         <v>5</v>
       </c>
       <c r="B128" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C128" s="17">
-        <v>672</v>
+        <v>423</v>
       </c>
       <c r="D128" s="19">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="E128" s="8" t="s">
         <v>1</v>
@@ -2688,13 +2688,13 @@
         <v>5</v>
       </c>
       <c r="B129" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C129" s="17">
-        <v>1929</v>
+        <v>672</v>
       </c>
       <c r="D129" s="19">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="E129" s="8" t="s">
         <v>1</v>
@@ -2705,13 +2705,13 @@
         <v>5</v>
       </c>
       <c r="B130" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C130" s="17">
-        <v>1087</v>
+        <v>1929</v>
       </c>
       <c r="D130" s="19">
-        <v>20500</v>
+        <v>14000</v>
       </c>
       <c r="E130" s="8" t="s">
         <v>1</v>
@@ -2722,13 +2722,13 @@
         <v>5</v>
       </c>
       <c r="B131" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C131" s="17">
-        <v>3179</v>
+        <v>1087</v>
       </c>
       <c r="D131" s="19">
-        <v>16500</v>
+        <v>16000</v>
       </c>
       <c r="E131" s="8" t="s">
         <v>1</v>
@@ -2736,16 +2736,16 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B132" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C132" s="17">
-        <v>1954</v>
+        <v>3179</v>
       </c>
       <c r="D132" s="19">
-        <v>84000</v>
+        <v>14000</v>
       </c>
       <c r="E132" s="8" t="s">
         <v>1</v>
@@ -2756,13 +2756,13 @@
         <v>6</v>
       </c>
       <c r="B133" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C133" s="17">
-        <v>1312</v>
+        <v>1954</v>
       </c>
       <c r="D133" s="19">
-        <v>47000</v>
+        <v>35000</v>
       </c>
       <c r="E133" s="8" t="s">
         <v>1</v>
@@ -2773,13 +2773,13 @@
         <v>6</v>
       </c>
       <c r="B134" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C134" s="17">
-        <v>874</v>
+        <v>1312</v>
       </c>
       <c r="D134" s="19">
-        <v>94000</v>
+        <v>40000</v>
       </c>
       <c r="E134" s="8" t="s">
         <v>1</v>
@@ -2787,19 +2787,19 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B135" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C135" s="17">
-        <v>1899</v>
+        <v>874</v>
       </c>
       <c r="D135" s="19">
-        <v>15000</v>
+        <v>40000</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
@@ -2807,13 +2807,13 @@
         <v>7</v>
       </c>
       <c r="B136" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C136" s="17">
-        <v>2985</v>
+        <v>1899</v>
       </c>
       <c r="D136" s="19">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="E136" s="8" t="s">
         <v>3</v>
@@ -2824,13 +2824,13 @@
         <v>7</v>
       </c>
       <c r="B137" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C137" s="17">
-        <v>2184</v>
+        <v>2985</v>
       </c>
       <c r="D137" s="19">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E137" s="8" t="s">
         <v>3</v>
@@ -2841,13 +2841,13 @@
         <v>7</v>
       </c>
       <c r="B138" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C138" s="17">
-        <v>519</v>
+        <v>2184</v>
       </c>
       <c r="D138" s="19">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="E138" s="8" t="s">
         <v>3</v>
@@ -2858,13 +2858,13 @@
         <v>7</v>
       </c>
       <c r="B139" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C139" s="17">
-        <v>2183</v>
+        <v>519</v>
       </c>
       <c r="D139" s="19">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E139" s="8" t="s">
         <v>3</v>
@@ -2875,13 +2875,13 @@
         <v>7</v>
       </c>
       <c r="B140" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C140" s="17">
-        <v>1884</v>
+        <v>2183</v>
       </c>
       <c r="D140" s="19">
-        <v>16000</v>
+        <v>10000</v>
       </c>
       <c r="E140" s="8" t="s">
         <v>3</v>
@@ -2892,13 +2892,13 @@
         <v>7</v>
       </c>
       <c r="B141" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C141" s="17">
-        <v>2185</v>
+        <v>1884</v>
       </c>
       <c r="D141" s="19">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="E141" s="8" t="s">
         <v>3</v>
@@ -2909,13 +2909,13 @@
         <v>7</v>
       </c>
       <c r="B142" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C142" s="17">
-        <v>1885</v>
+        <v>2185</v>
       </c>
       <c r="D142" s="19">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="E142" s="8" t="s">
         <v>3</v>
@@ -2926,13 +2926,13 @@
         <v>7</v>
       </c>
       <c r="B143" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C143" s="17">
-        <v>3389</v>
+        <v>1885</v>
       </c>
       <c r="D143" s="19">
-        <v>8000</v>
+        <v>13000</v>
       </c>
       <c r="E143" s="8" t="s">
         <v>3</v>
@@ -2943,13 +2943,13 @@
         <v>7</v>
       </c>
       <c r="B144" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C144" s="17">
-        <v>1883</v>
+        <v>3389</v>
       </c>
       <c r="D144" s="19">
-        <v>16000</v>
+        <v>8000</v>
       </c>
       <c r="E144" s="8" t="s">
         <v>3</v>
@@ -2957,19 +2957,19 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B145" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C145" s="17">
-        <v>2476</v>
+        <v>1883</v>
       </c>
       <c r="D145" s="19">
-        <v>1490</v>
+        <v>12000</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
@@ -2977,13 +2977,13 @@
         <v>9</v>
       </c>
       <c r="B146" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C146" s="17">
-        <v>2494</v>
+        <v>2476</v>
       </c>
       <c r="D146" s="19">
-        <v>1412</v>
+        <v>1490</v>
       </c>
       <c r="E146" s="8" t="s">
         <v>4</v>
@@ -2994,13 +2994,13 @@
         <v>9</v>
       </c>
       <c r="B147" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C147" s="17">
-        <v>2661</v>
+        <v>2494</v>
       </c>
       <c r="D147" s="19">
-        <v>1257</v>
+        <v>1412</v>
       </c>
       <c r="E147" s="8" t="s">
         <v>4</v>
@@ -3011,13 +3011,13 @@
         <v>9</v>
       </c>
       <c r="B148" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C148" s="17">
-        <v>3465</v>
+        <v>2661</v>
       </c>
       <c r="D148" s="19">
-        <v>714</v>
+        <v>1257</v>
       </c>
       <c r="E148" s="8" t="s">
         <v>4</v>
@@ -3028,10 +3028,10 @@
         <v>9</v>
       </c>
       <c r="B149" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C149" s="17">
-        <v>1133</v>
+        <v>3465</v>
       </c>
       <c r="D149" s="19">
         <v>714</v>
@@ -3045,10 +3045,10 @@
         <v>9</v>
       </c>
       <c r="B150" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C150" s="17">
-        <v>3467</v>
+        <v>1133</v>
       </c>
       <c r="D150" s="19">
         <v>714</v>
@@ -3059,16 +3059,16 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B151" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C151" s="17">
-        <v>1762</v>
+        <v>3467</v>
       </c>
       <c r="D151" s="19">
-        <v>42853</v>
+        <v>714</v>
       </c>
       <c r="E151" s="8" t="s">
         <v>4</v>
@@ -3079,13 +3079,13 @@
         <v>8</v>
       </c>
       <c r="B152" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C152" s="17">
-        <v>1778</v>
+        <v>1762</v>
       </c>
       <c r="D152" s="19">
-        <v>33671</v>
+        <v>42853</v>
       </c>
       <c r="E152" s="8" t="s">
         <v>4</v>
@@ -3096,13 +3096,13 @@
         <v>8</v>
       </c>
       <c r="B153" s="15">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="C153" s="17">
-        <v>2727</v>
+        <v>1778</v>
       </c>
       <c r="D153" s="19">
-        <v>29079</v>
+        <v>40707</v>
       </c>
       <c r="E153" s="8" t="s">
         <v>4</v>
@@ -3110,868 +3110,18 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B154" s="15">
         <v>46266</v>
       </c>
       <c r="C154" s="17">
-        <v>27</v>
+        <v>2727</v>
       </c>
       <c r="D154" s="19">
-        <v>310000</v>
+        <v>39634</v>
       </c>
       <c r="E154" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A155" s="5">
-        <v>1</v>
-      </c>
-      <c r="B155" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C155" s="7">
-        <v>1139</v>
-      </c>
-      <c r="D155" s="4">
-        <v>320000</v>
-      </c>
-      <c r="E155" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A156" s="5">
-        <v>1</v>
-      </c>
-      <c r="B156" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C156" s="7">
-        <v>675</v>
-      </c>
-      <c r="D156" s="4">
-        <v>210000</v>
-      </c>
-      <c r="E156" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A157" s="5">
-        <v>1</v>
-      </c>
-      <c r="B157" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C157" s="7">
-        <v>58</v>
-      </c>
-      <c r="D157" s="4">
-        <v>170000</v>
-      </c>
-      <c r="E157" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A158" s="5">
-        <v>1</v>
-      </c>
-      <c r="B158" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C158" s="7">
-        <v>841</v>
-      </c>
-      <c r="D158" s="4">
-        <v>100000</v>
-      </c>
-      <c r="E158" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A159" s="5">
-        <v>1</v>
-      </c>
-      <c r="B159" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C159" s="7">
-        <v>13148</v>
-      </c>
-      <c r="D159" s="4">
-        <v>150000</v>
-      </c>
-      <c r="E159" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A160" s="5">
-        <v>1</v>
-      </c>
-      <c r="B160" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C160" s="7">
-        <v>805</v>
-      </c>
-      <c r="D160" s="4">
-        <v>300000</v>
-      </c>
-      <c r="E160" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A161" s="5">
-        <v>1</v>
-      </c>
-      <c r="B161" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C161" s="7">
-        <v>3403</v>
-      </c>
-      <c r="D161" s="4">
-        <v>250000</v>
-      </c>
-      <c r="E161" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A162" s="5">
-        <v>2</v>
-      </c>
-      <c r="B162" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C162" s="7">
-        <v>1898</v>
-      </c>
-      <c r="D162" s="4">
-        <v>250000</v>
-      </c>
-      <c r="E162" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A163" s="5">
-        <v>2</v>
-      </c>
-      <c r="B163" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C163" s="7">
-        <v>546</v>
-      </c>
-      <c r="D163" s="4">
-        <v>260000</v>
-      </c>
-      <c r="E163" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A164" s="5">
-        <v>2</v>
-      </c>
-      <c r="B164" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C164" s="7">
-        <v>422</v>
-      </c>
-      <c r="D164" s="4">
-        <v>260000</v>
-      </c>
-      <c r="E164" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A165" s="5">
-        <v>2</v>
-      </c>
-      <c r="B165" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C165" s="7">
-        <v>1281</v>
-      </c>
-      <c r="D165" s="4">
-        <v>280000</v>
-      </c>
-      <c r="E165" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A166" s="5">
-        <v>2</v>
-      </c>
-      <c r="B166" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C166" s="7">
-        <v>2220</v>
-      </c>
-      <c r="D166" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E166" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A167" s="5">
-        <v>2</v>
-      </c>
-      <c r="B167" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C167" s="7">
-        <v>2571</v>
-      </c>
-      <c r="D167" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E167" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A168" s="5">
-        <v>3</v>
-      </c>
-      <c r="B168" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C168" s="7">
-        <v>2845</v>
-      </c>
-      <c r="D168" s="4">
-        <v>100000</v>
-      </c>
-      <c r="E168" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A169" s="5">
-        <v>3</v>
-      </c>
-      <c r="B169" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C169" s="7">
-        <v>691</v>
-      </c>
-      <c r="D169" s="4">
-        <v>250000</v>
-      </c>
-      <c r="E169" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A170" s="5">
-        <v>3</v>
-      </c>
-      <c r="B170" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C170" s="7">
-        <v>1533</v>
-      </c>
-      <c r="D170" s="4">
-        <v>340000</v>
-      </c>
-      <c r="E170" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A171" s="5">
-        <v>3</v>
-      </c>
-      <c r="B171" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C171" s="7">
-        <v>738</v>
-      </c>
-      <c r="D171" s="4">
-        <v>220000</v>
-      </c>
-      <c r="E171" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A172" s="5">
-        <v>3</v>
-      </c>
-      <c r="B172" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C172" s="7">
-        <v>213</v>
-      </c>
-      <c r="D172" s="4">
-        <v>80000</v>
-      </c>
-      <c r="E172" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A173" s="5">
-        <v>3</v>
-      </c>
-      <c r="B173" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C173" s="7">
-        <v>3009</v>
-      </c>
-      <c r="D173" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E173" s="8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A174" s="5">
-        <v>4</v>
-      </c>
-      <c r="B174" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C174" s="7">
-        <v>3449</v>
-      </c>
-      <c r="D174" s="4">
-        <v>230000</v>
-      </c>
-      <c r="E174" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A175" s="5">
-        <v>4</v>
-      </c>
-      <c r="B175" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C175" s="7">
-        <v>1953</v>
-      </c>
-      <c r="D175" s="4">
-        <v>220000</v>
-      </c>
-      <c r="E175" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A176" s="5">
-        <v>4</v>
-      </c>
-      <c r="B176" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C176" s="7">
-        <v>2853</v>
-      </c>
-      <c r="D176" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E176" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A177" s="5">
-        <v>5</v>
-      </c>
-      <c r="B177" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C177" s="7">
-        <v>977</v>
-      </c>
-      <c r="D177" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E177" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A178" s="5">
-        <v>5</v>
-      </c>
-      <c r="B178" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C178" s="7">
-        <v>423</v>
-      </c>
-      <c r="D178" s="4">
-        <v>250000</v>
-      </c>
-      <c r="E178" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A179" s="5">
-        <v>5</v>
-      </c>
-      <c r="B179" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C179" s="7">
-        <v>672</v>
-      </c>
-      <c r="D179" s="4">
-        <v>250000</v>
-      </c>
-      <c r="E179" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A180" s="5">
-        <v>5</v>
-      </c>
-      <c r="B180" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C180" s="7">
-        <v>1929</v>
-      </c>
-      <c r="D180" s="4">
-        <v>210000</v>
-      </c>
-      <c r="E180" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A181" s="5">
-        <v>5</v>
-      </c>
-      <c r="B181" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C181" s="7">
-        <v>1087</v>
-      </c>
-      <c r="D181" s="4">
-        <v>170000</v>
-      </c>
-      <c r="E181" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A182" s="5">
-        <v>5</v>
-      </c>
-      <c r="B182" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C182" s="7">
-        <v>3179</v>
-      </c>
-      <c r="D182" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E182" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A183" s="5">
-        <v>6</v>
-      </c>
-      <c r="B183" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C183" s="7">
-        <v>1954</v>
-      </c>
-      <c r="D183" s="4">
-        <v>180000</v>
-      </c>
-      <c r="E183" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A184" s="5">
-        <v>6</v>
-      </c>
-      <c r="B184" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C184" s="7">
-        <v>1312</v>
-      </c>
-      <c r="D184" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E184" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A185" s="5">
-        <v>6</v>
-      </c>
-      <c r="B185" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C185" s="7">
-        <v>874</v>
-      </c>
-      <c r="D185" s="4">
-        <v>200000</v>
-      </c>
-      <c r="E185" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A186" s="5">
-        <v>7</v>
-      </c>
-      <c r="B186" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C186" s="7">
-        <v>1899</v>
-      </c>
-      <c r="D186" s="4">
-        <v>245000</v>
-      </c>
-      <c r="E186" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A187" s="5">
-        <v>7</v>
-      </c>
-      <c r="B187" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C187" s="7">
-        <v>2985</v>
-      </c>
-      <c r="D187" s="4">
-        <v>126000</v>
-      </c>
-      <c r="E187" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A188" s="5">
-        <v>7</v>
-      </c>
-      <c r="B188" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C188" s="7">
-        <v>2184</v>
-      </c>
-      <c r="D188" s="4">
-        <v>195000</v>
-      </c>
-      <c r="E188" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A189" s="5">
-        <v>7</v>
-      </c>
-      <c r="B189" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C189" s="7">
-        <v>519</v>
-      </c>
-      <c r="D189" s="4">
-        <v>360000</v>
-      </c>
-      <c r="E189" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A190" s="5">
-        <v>7</v>
-      </c>
-      <c r="B190" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C190" s="7">
-        <v>2183</v>
-      </c>
-      <c r="D190" s="4">
-        <v>136000</v>
-      </c>
-      <c r="E190" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A191" s="5">
-        <v>7</v>
-      </c>
-      <c r="B191" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C191" s="7">
-        <v>1884</v>
-      </c>
-      <c r="D191" s="4">
-        <v>195000</v>
-      </c>
-      <c r="E191" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A192" s="5">
-        <v>7</v>
-      </c>
-      <c r="B192" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C192" s="7">
-        <v>2185</v>
-      </c>
-      <c r="D192" s="4">
-        <v>136000</v>
-      </c>
-      <c r="E192" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A193" s="5">
-        <v>7</v>
-      </c>
-      <c r="B193" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C193" s="7">
-        <v>1885</v>
-      </c>
-      <c r="D193" s="4">
-        <v>160000</v>
-      </c>
-      <c r="E193" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A194" s="5">
-        <v>7</v>
-      </c>
-      <c r="B194" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C194" s="7">
-        <v>3389</v>
-      </c>
-      <c r="D194" s="4">
-        <v>96000</v>
-      </c>
-      <c r="E194" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A195" s="5">
-        <v>7</v>
-      </c>
-      <c r="B195" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C195" s="7">
-        <v>1883</v>
-      </c>
-      <c r="D195" s="4">
-        <v>210000</v>
-      </c>
-      <c r="E195" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A196" s="5">
-        <v>9</v>
-      </c>
-      <c r="B196" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C196" s="7">
-        <v>2476</v>
-      </c>
-      <c r="D196" s="4">
-        <v>190000</v>
-      </c>
-      <c r="E196" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A197" s="5">
-        <v>9</v>
-      </c>
-      <c r="B197" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C197" s="7">
-        <v>2494</v>
-      </c>
-      <c r="D197" s="4">
-        <v>150000</v>
-      </c>
-      <c r="E197" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A198" s="5">
-        <v>9</v>
-      </c>
-      <c r="B198" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C198" s="7">
-        <v>2661</v>
-      </c>
-      <c r="D198" s="4">
-        <v>125000</v>
-      </c>
-      <c r="E198" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A199" s="5">
-        <v>9</v>
-      </c>
-      <c r="B199" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C199" s="7">
-        <v>3465</v>
-      </c>
-      <c r="D199" s="4">
-        <v>115667</v>
-      </c>
-      <c r="E199" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A200" s="5">
-        <v>9</v>
-      </c>
-      <c r="B200" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C200" s="7">
-        <v>1133</v>
-      </c>
-      <c r="D200" s="4">
-        <v>115667</v>
-      </c>
-      <c r="E200" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A201" s="5">
-        <v>9</v>
-      </c>
-      <c r="B201" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C201" s="7">
-        <v>3467</v>
-      </c>
-      <c r="D201" s="4">
-        <v>115667</v>
-      </c>
-      <c r="E201" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A202" s="5">
-        <v>8</v>
-      </c>
-      <c r="B202" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C202" s="7">
-        <v>1762</v>
-      </c>
-      <c r="D202" s="4">
-        <v>280000</v>
-      </c>
-      <c r="E202" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A203" s="5">
-        <v>8</v>
-      </c>
-      <c r="B203" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C203" s="7">
-        <v>1778</v>
-      </c>
-      <c r="D203" s="4">
-        <v>265978</v>
-      </c>
-      <c r="E203" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A204" s="5">
-        <v>8</v>
-      </c>
-      <c r="B204" s="2">
-        <v>46266</v>
-      </c>
-      <c r="C204" s="7">
-        <v>2727</v>
-      </c>
-      <c r="D204" s="4">
-        <v>190000</v>
-      </c>
-      <c r="E204" s="8" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>